<commit_message>
BH ledger: import derived-1/4, add prediction column, fix 042/043
- Port BH_Thermal2Pi_EntropyCoefficient into EDG (geometric derivation of
  the Bekenstein-Hawking 1/4 from ED's own near-horizon Rindler geometry;
  Euclidean-continuation tool, on par with GR; arrow-native 2pi OPEN per its
  own honest 4b negative). Net folder status of the 1/4 flips INHERITED ->
  DERIVED; resolves the README-vs-043 tension (ledger Staleness #1).
- Master xlsx: add 'Falsifier / Kill-Cond' column tying predictions to their
  kill-conditions (merger-lag -> 22-Ways P2, provisional). Deterministic full
  rebuild so changed rows leave no orphans. 55 rows.
- 042: 'C_max ~ r^3/l_P^3 (P04-derived)' -> posited (P-Bandwidth-Boundedness);
  note the bottom-up P04 derivation failed (FiniteGrain lemma).
- 043: stale Paper_067 refs -> Paper_068 (superseded 2026-07-05).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ED_TieredClaims_Master.xlsx
+++ b/ED_TieredClaims_Master.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Claims" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Claims'!$A$1:$H$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Claims'!$A$1:$I$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -450,17 +450,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,20 +487,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Falsifier / Kill-Cond</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Derived</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Inherited/Open</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>SpotChecked</t>
         </is>
@@ -513,33 +519,38 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>043</t>
+          <t>BH_Thermal2Pi</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Bekenstein-Hawking 1/4 coefficient</t>
+          <t>Bekenstein-Hawking coefficient 1/4 (T=kappa/2pi, S=A/4), GEOMETRIC route</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Selected/Inherited</t>
+          <t>Derived</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>I — via log-g matching (log g = pi); 'matching, not derivation' (§4, conclusion)</t>
+          <t>Both factors ED-structural: 1/2 from kappa=1/(2r_s) (b-profile slope, GR-III); 2pi from near-horizon Rindler shape via smoothness (numerically confirmed)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>current — in-folder EDG status of the 1/4 is INHERITED (Staleness #1)</t>
+          <t>tool = Euclidean continuation, the SAME route GR uses (on par with GR, not beyond); b-profile + kappa inherited from GR-III; arrow-native continuation-free 2pi OPEN (§4b)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>yes 2026-07-29</t>
+          <t>current — the in-folder DERIVED route for the 1/4 (imported 2026-07-29)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-29 (read in full before import)</t>
         </is>
       </c>
     </row>
@@ -551,31 +562,40 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>044_5</t>
+          <t>039</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Greybody factors Gamma_ls</t>
+          <t>Horizon = b-&gt;0 decoupling surface (Gamma_cross collapse)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Selected/Inherited</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>I — 'NOT a new derivation... INHERITED from Regge-Wheeler 1957/Zerilli/Page'</t>
+          <t>D mechanism (decoupling-surface)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>r_H location + kappa INHERITED from GR (§3.2 honest-ack: r_H a CG reference, not derived)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-29</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -585,31 +605,36 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>047_5</t>
+          <t>040</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Universal T = kappa/2pi for all 4 horizon types</t>
+          <t>Trans-Planckian resolution (modes terminate at wc)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Selected/Inherited</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>I — 'INHERITED from standard semi-classical GR'; genuine ED content = V5-saturation identification only</t>
+          <t>D-via-I</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
+          <t>conditional on P-V5-UV-Cutoff + P-Cutoff-Saturation</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -619,31 +644,36 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>050</t>
+          <t>041</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>t_Page ~ 0.54·tau_BH; c1, wc, c* values</t>
+          <t>Planck-mass remnant M* = c*·l_P (Scenario C)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Selected/Inherited</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>D-via-I</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr"/>
+          <t>conditional on P-Cutoff-Saturation-Endpoint + P-Remnant-Stability + 048; c* inherited</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -653,31 +683,40 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>041</t>
+          <t>042</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>'Remnants NOT a dark-matter candidate'</t>
+          <t>No-singularity (C_cum bounded, r &gt;= l_P)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Asserted</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>A-&gt;position</t>
+          <t>D-via-I</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
+          <t>conditional on P-Bandwidth-Boundedness + P-Substrate-Interior-Cutoff; interior OPEN</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>current — abstract's 'P04-derived' is really postulated (Staleness #3)</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-29</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -687,31 +726,36 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>042</t>
+          <t>043</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>'Classical singularity is a coarse-graining artifact'</t>
+          <t>Area-law FORM S ∝ A</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Asserted</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>A-&gt;position</t>
+          <t>D-via-I (form forced)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
+          <t>conditional on P-Horizon-Participation + P-Multiplicity-g; coefficient inherited by this route</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>current (the FORM; coefficient has a separate geometric route — next row)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -721,31 +765,36 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>044_5</t>
+          <t>044</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>'Leading-order match is identification, not derivation'</t>
+          <t>BHPT scattering / Regge-Wheeler form</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Asserted</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>A-&gt;position; greybody factors inherited</t>
+          <t>form-forced</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
+          <t>conditional on P-Horizon-Ingoing-Only + P-Asymptotic-Outgoing; cross-sections inherited</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -755,31 +804,36 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>047_5</t>
+          <t>045</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>'Four-horizon structural identification'</t>
+          <t>Helicity preserved (Schwarzschild) / amplified (Kerr)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Asserted</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>A-&gt;position; temperature fully inherited</t>
+          <t>form-forced</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
+          <t>conditional on P-Helicity-Channel + P-Kerr-Helicity-Coupling; superradiance OPEN</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -789,35 +843,36 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>051</t>
+          <t>046</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>'Paradox not generated' + 'information not lost'</t>
+          <t>Kerr twist g_tphi</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Asserted</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>A-&gt;position (audit rows 9-10); rests on P-Substrate-Unitarity; 'structural ledger, not constructive proof'</t>
+          <t>form-forced</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>current — the arc's load-bearing soft spot</t>
+          <t>conditional on P-Substrate-Vorticity + P-Twist-Coarse-Graining; a inherited; interior OPEN</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>yes 2026-07-29</t>
-        </is>
-      </c>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -827,31 +882,36 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>047_5</t>
+          <t>047</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Cross-class horizon identification (M3)</t>
+          <t>Hawking temperature T_H = kappa/2pi via V5 KMS</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Synthesis</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>genuine ED content = the V5-saturation mechanism only</t>
+          <t>KMS =&gt; thermal = D</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
+          <t>kappa I; Euclidean/conical 2pi = I-via-DCGT (audit rows 5-8, not substrate-derived)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>current — see Staleness #2 on the '2pi derived' claim</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -861,31 +921,36 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>052</t>
+          <t>047</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Paradox synthesis (integrates 039+047+050+041)</t>
+          <t>Non-thermal Hawking correction [1 - c1(w/wc)^2]</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Synthesis</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>arc consolidation</t>
+          <t>D form</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
+          <t>conditional on P-V5-Even; wc chosen-to-match, c1 inherited</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -895,31 +960,36 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>042/046</t>
+          <t>048</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Substrate BH interior for r &lt; l_P</t>
+          <t>Scenario C forced (A, B excluded)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>D-via-I</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
+          <t>conditional on P-Resummation-Convergence + P-Endpoint-Truncation; coeffs inherited</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -929,31 +999,36 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>043</t>
+          <t>049</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Substrate derivation of log g</t>
+          <t>PBH relic abundance Omega* ∝ n_PBH·M*</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>D-via-I</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
+          <t>conditional on P-One-Remnant-Per-PBH</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -963,31 +1038,36 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>045</t>
+          <t>050</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Superradiance</t>
+          <t>Page-curve rise + turnover + decline</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>D-via-I / Form-forced</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
+          <t>conditional on P-V5-EntBudget + P-Re-routing; t_Page ~ 0.54·tau_BH inherited; unitarity OPEN</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -997,31 +1077,40 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>047/BH_Thermal2Pi</t>
+          <t>HorizonTiling</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Arrow-native (continuation-free) 2pi</t>
+          <t>Horizon tiles ~1 bit/Planck cell (3 counts: holo=1, frozen 0.78, edge 0.88)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Measured</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>OPEN — the derived-2pi route is Euclidean (reversible-time); arrow-native 2pi not yet supplied</t>
+          <t>measured convergence</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>open (memo relocated OUT of EDG)</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
+          <t>2 of 3 counts assume the emergent geometry (curvature emergence OPEN); scale l_V5~l_P inherited</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>current — explicit consilience, 'not a novel prediction, not tiered as one'</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-29</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1031,31 +1120,36 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>050/051</t>
+          <t>043</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Full unitarity (constructive, not postulated)</t>
+          <t>Bekenstein-Hawking 1/4 coefficient, COMBINATORIAL route</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Selected/Inherited</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>OPEN — target #4; 051 assumes it (P-Substrate-Unitarity)</t>
-        </is>
-      </c>
+      <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr"/>
+          <t>I — via log-g matching (log g = pi); 'matching, not derivation' (§4). NOTE: folder also has the geometric DERIVED route (BH_Thermal2Pi); net folder status of the 1/4 = DERIVED</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>current — this route inherits; net 1/4 now derived (Staleness #1 RESOLVED)</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-29</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1065,31 +1159,32 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>052_5</t>
+          <t>044_5</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Substrate-anchored tau_V5 floor (merger-lag)</t>
+          <t>Greybody factors Gamma_ls</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Selected/Inherited</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
+      <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>I — 'NOT a new derivation... INHERITED from Regge-Wheeler 1957/Zerilli/Page'</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1099,31 +1194,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>HorizonTiling/046</t>
+          <t>047_5</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Curvature emergence underneath the geometric counts</t>
+          <t>Universal T = kappa/2pi for all 4 horizon types</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Selected/Inherited</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>OPEN — the bridge under 2-of-3 tiling counts + the Kerr geometry</t>
-        </is>
-      </c>
+      <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
+          <t>I — 'INHERITED from standard semi-classical GR'; genuine ED content = V5-saturation identification only</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1133,39 +1229,32 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>039</t>
+          <t>050</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Horizon = b-&gt;0 decoupling surface (Gamma_cross collapse)</t>
+          <t>t_Page ~ 0.54·tau_BH; c1, wc, c* values</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>D mechanism (decoupling-surface)</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>r_H location + kappa INHERITED from GR (§3.2 honest-ack: r_H a CG reference, not derived)</t>
-        </is>
-      </c>
+          <t>Selected/Inherited</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>current</t>
+          <t>I</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>yes 2026-07-29</t>
-        </is>
-      </c>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1175,35 +1264,32 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>040</t>
+          <t>041</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Trans-Planckian resolution (modes terminate at wc)</t>
+          <t>'Remnants NOT a dark-matter candidate'</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>D-via-I</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-V5-UV-Cutoff + P-Cutoff-Saturation</t>
-        </is>
-      </c>
+          <t>Asserted</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
+          <t>A-&gt;position</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1213,35 +1299,32 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>041</t>
+          <t>042</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Planck-mass remnant M* = c*·l_P (Scenario C)</t>
+          <t>'Classical singularity is a coarse-graining artifact'</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>D-via-I</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-Cutoff-Saturation-Endpoint + P-Remnant-Stability + 048; c* inherited</t>
-        </is>
-      </c>
+          <t>Asserted</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>A-&gt;position</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1251,39 +1334,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>042</t>
+          <t>044_5</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>No-singularity (C_cum bounded, r &gt;= l_P)</t>
+          <t>'Leading-order match is identification, not derivation'</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>D-via-I</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-Bandwidth-Boundedness + P-Substrate-Interior-Cutoff; interior OPEN</t>
-        </is>
-      </c>
+          <t>Asserted</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>current — abstract's 'P04-derived' is really postulated (Staleness #3)</t>
+          <t>A-&gt;position; greybody factors inherited</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>yes 2026-07-29</t>
-        </is>
-      </c>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1293,35 +1369,32 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>043</t>
+          <t>047_5</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Area-law FORM S ∝ A</t>
+          <t>'Four-horizon structural identification'</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>D-via-I (form forced)</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-Horizon-Participation + P-Multiplicity-g; coefficient inherited</t>
-        </is>
-      </c>
+          <t>Asserted</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>current (the FORM; coefficient separate — Staleness #1)</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>A-&gt;position; temperature fully inherited</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1331,35 +1404,36 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>044</t>
+          <t>051</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>BHPT scattering / Regge-Wheeler form</t>
+          <t>'Paradox not generated' + 'information not lost'</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>form-forced</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-Horizon-Ingoing-Only + P-Asymptotic-Outgoing; cross-sections inherited</t>
-        </is>
-      </c>
+          <t>Asserted</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr"/>
+          <t>A-&gt;position (audit rows 9-10); rests on P-Substrate-Unitarity; 'structural ledger, not constructive proof'</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>current — the arc's load-bearing soft spot</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-29</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1369,35 +1443,40 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>045</t>
+          <t>052_5</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Helicity preserved (Schwarzschild) / amplified (Kerr)</t>
+          <t>Merger-lag (existence of a delay)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
+          <t>Prediction</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>form-forced</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-Helicity-Channel + P-Kerr-Helicity-Coupling; superradiance OPEN</t>
-        </is>
-      </c>
+          <t>22-Ways P2 (merger-lag): PROVISIONAL, existence-only; NOT refutation-grade (needs substrate tau_V5 floor, OPEN)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
+          <t>PROVISIONAL / M2, existence-only; tau_V5 floor OPEN; numerics inherited; zero D rows (row 14 A-&gt;position); NOT refutation-grade in BTFR sense; confirms 22-Ways P2</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>current — do not upgrade until a substrate tau_V5 floor is supplied</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-29</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1407,35 +1486,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>046</t>
+          <t>047_5</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Kerr twist g_tphi</t>
+          <t>Cross-class horizon identification (M3)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>form-forced</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-Substrate-Vorticity + P-Twist-Coarse-Graining; a inherited; interior OPEN</t>
-        </is>
-      </c>
+          <t>Synthesis</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr"/>
+          <t>genuine ED content = the V5-saturation mechanism only</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1445,35 +1521,32 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>047</t>
+          <t>052</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Hawking temperature T_H = kappa/2pi via V5 KMS</t>
+          <t>Paradox synthesis (integrates 039+047+050+041)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>KMS =&gt; thermal = D</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>kappa I; Euclidean/conical 2pi = I-via-DCGT (audit rows 5-8, not substrate-derived)</t>
-        </is>
-      </c>
+          <t>Synthesis</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>current — see Staleness #2 on the '2pi derived' claim</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
+          <t>arc consolidation</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1483,35 +1556,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>047</t>
+          <t>042/046</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Non-thermal Hawking correction [1 - c1(w/wc)^2]</t>
+          <t>Substrate BH interior for r &lt; l_P</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>D form</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-V5-Even; wc chosen-to-match, c1 inherited</t>
-        </is>
-      </c>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr"/>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1521,35 +1591,32 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>048</t>
+          <t>043</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Scenario C forced (A, B excluded)</t>
+          <t>Substrate derivation of log g</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>D-via-I</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-Resummation-Convergence + P-Endpoint-Truncation; coeffs inherited</t>
-        </is>
-      </c>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1559,35 +1626,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>049</t>
+          <t>045</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>PBH relic abundance Omega* ∝ n_PBH·M*</t>
+          <t>Superradiance</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>D-via-I</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-One-Remnant-Per-PBH</t>
-        </is>
-      </c>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1597,35 +1661,32 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>050</t>
+          <t>050/051</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Page-curve rise + turnover + decline</t>
+          <t>Full unitarity (constructive, not postulated)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>D-via-I / Form-forced</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-V5-EntBudget + P-Re-routing; t_Page ~ 0.54·tau_BH inherited; unitarity OPEN</t>
-        </is>
-      </c>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
+          <t>OPEN — target #4; 051 assumes it (P-Substrate-Unitarity)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1640,30 +1701,31 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Merger-lag (existence of a delay)</t>
+          <t>Substrate-anchored tau_V5 floor (merger-lag)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Prediction</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>PROVISIONAL / M2, existence-only; tau_V5 floor OPEN; numerics inherited; zero D rows (row 14 A-&gt;position); NOT refutation-grade in BTFR sense; confirms 22-Ways P2</t>
-        </is>
-      </c>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>22-Ways P2 (merger-lag): PROVISIONAL, existence-only; NOT refutation-grade (needs substrate tau_V5 floor, OPEN)</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>current — do not upgrade until a substrate tau_V5 floor is supplied</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>yes 2026-07-29</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1673,75 +1735,67 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>HorizonTiling</t>
+          <t>BH_Thermal2Pi</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Horizon tiles ~1 bit/Planck cell (3 counts: holo=1, frozen 0.78, edge 0.88)</t>
+          <t>Arrow-native (continuation-free) 2pi</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Measured</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>measured convergence</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>2 of 3 counts assume the emergent geometry (curvature emergence OPEN); scale l_V5~l_P inherited</t>
-        </is>
-      </c>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>current — explicit consilience, 'not a novel prediction, not tiered as one'</t>
+          <t>OPEN — derived-2pi route is Euclidean (reversible-time), on par with GR; arrow-native 2pi from raw commitment statistics not yet supplied (§4b honest negative; possibly a category error — 2pi may be an intrinsically continuum feature)</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>yes 2026-07-29</t>
-        </is>
-      </c>
+          <t>open (§4b, now in-folder)</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Entanglement</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>64</v>
+          <t>Black-hole</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>HorizonTiling/046</t>
+        </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Schmidt rank&gt;1 =&gt; non-factorizable</t>
+          <t>Curvature emergence underneath the geometric counts</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>D (standard SVD applied)</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>conditional on P-V5-Schmidt-Generic</t>
-        </is>
-      </c>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>current — strengthens 063 only under that postulate</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr"/>
+          <t>OPEN — the bridge under 2-of-3 tiling counts + the Kerr geometry</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1749,12 +1803,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
-        <v>65</v>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>064</t>
+        </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Monogamy (CKW-form inequality)</t>
+          <t>Schmidt rank&gt;1 =&gt; non-factorizable</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1762,22 +1818,23 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>form D (form-forced) from V5 finite budget + P04 additivity</t>
-        </is>
-      </c>
+      <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>conditional on P-V5-Budget + P-Measure-Saturation; coefficient inherited</t>
+          <t>D (standard SVD applied)</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr"/>
+          <t>conditional on P-V5-Schmidt-Generic</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>current — strengthens 063 only under that postulate</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1785,12 +1842,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
-        <v>66</v>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>065</t>
+        </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>No-signaling p(a|x,y)=p(a|x), over-determined by 3 locks</t>
+          <t>Monogamy (CKW-form inequality)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1798,26 +1857,23 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Lock L1 (marginal independence) = D-via-I from tensor-product + POVM completeness</t>
-        </is>
-      </c>
+      <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>L2 rests on P-Substrate-Causality; L3 = Paper_073; '3-locks =&gt; over-determination' is A-&gt;position</t>
+          <t>form D (form-forced) from V5 finite budget + P04 additivity</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>current — cleanest paper in arc; Bell-Tsirelson explicitly OPEN here (row 11)</t>
+          <t>conditional on P-V5-Budget + P-Measure-Saturation; coefficient inherited</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>yes 2026-07-28</t>
-        </is>
-      </c>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1825,12 +1881,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B38" s="2" t="n">
-        <v>68</v>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>066</t>
+        </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>von Neumann entropy form S = -Tr rho log rho</t>
+          <t>No-signaling p(a|x,y)=p(a|x), over-determined by 3 locks</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1838,22 +1896,27 @@
           <t>Derived</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>D-via-I (Shannon-Khinchin + Khinchin uniqueness)</t>
-        </is>
-      </c>
+      <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>conditional on P-Continuity + P-Additivity + P-Maximality; normalization inherited</t>
+          <t>Lock L1 (marginal independence) = D-via-I from tensor-product + POVM completeness</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>current — two substrate-derivations open</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr"/>
+          <t>L2 rests on P-Substrate-Causality; L3 = Paper_073; '3-locks =&gt; over-determination' is A-&gt;position</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>current — cleanest paper in arc; Bell-Tsirelson explicitly OPEN here (row 11)</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-28</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1861,35 +1924,38 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
-        <v>63</v>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>068</t>
+        </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>E-2 bilocal cross-chain term Delta_KL exists</t>
+          <t>von Neumann entropy form S = -Tr rho log rho</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Grounded</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>D conditional on V5 (Paper_090)</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr"/>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>D-via-I (Shannon-Khinchin + Khinchin uniqueness)</t>
+        </is>
+      </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>current</t>
+          <t>conditional on P-Continuity + P-Additivity + P-Maximality; normalization inherited</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>yes 2026-07-28</t>
-        </is>
-      </c>
+          <t>current — two substrate-derivations open</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1897,31 +1963,38 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
-        <v>64</v>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>063</t>
+        </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>The Schmidt decomposition form itself</t>
+          <t>E-2 bilocal cross-chain term Delta_KL exists</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Selected/Inherited</t>
+          <t>Grounded</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>I — SVD is standard math (round-7 relabel: was D-cond-SVD, now I)</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr"/>
+          <t>D conditional on V5 (Paper_090)</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-28</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1929,12 +2002,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B41" s="2" t="n">
-        <v>68</v>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>064</t>
+        </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>k_B / log-base normalization; concrete entropy values</t>
+          <t>The Schmidt decomposition form itself</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1943,17 +2018,18 @@
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
+      <c r="F41" s="2" t="inlineStr"/>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr"/>
+          <t>I — SVD is standard math (round-7 relabel: was D-cond-SVD, now I)</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1961,12 +2037,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n">
-        <v>69</v>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>068</t>
+        </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Tsirelson bound 2*sqrt(2)</t>
+          <t>k_B / log-base normalization; concrete entropy values</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1975,17 +2053,18 @@
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>I — 'not derived from first principles... INHERITED' (preamble 1)</t>
-        </is>
-      </c>
+      <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1993,12 +2072,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n">
-        <v>69</v>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>069</t>
+        </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Bell &lt; Tsirelson &lt; NS nesting; PR-box exclusion</t>
+          <t>Tsirelson bound 2*sqrt(2)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2006,26 +2087,19 @@
           <t>Selected/Inherited</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>D-via-I (form composition)</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>entirely conditional on P-V5-Hilbert-Constraint</t>
-        </is>
-      </c>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>current — inherits a Soler residual (see Status/staleness)</t>
+          <t>I — 'not derived from first principles... INHERITED' (preamble 1)</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>yes 2026-07-28</t>
-        </is>
-      </c>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2033,31 +2107,38 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B44" s="2" t="n">
-        <v>63</v>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>069</t>
+        </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>E-1 factorizable Psi^AB = Psi^A x Psi^B &amp; the tensor-product structure</t>
+          <t>Bell &lt; Tsirelson &lt; NS nesting; PR-box exclusion</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Postulated</t>
+          <t>Selected/Inherited</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>P-Bipartite-Mapping — 'definitional commitment, not a separate derivation'</t>
+          <t>D-via-I (form composition)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>current</t>
+          <t>entirely conditional on P-V5-Hilbert-Constraint</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>current — inherits a Soler residual (see Status/staleness)</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>yes 2026-07-28</t>
         </is>
@@ -2069,12 +2150,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B45" s="2" t="n">
-        <v>64</v>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>063</t>
+        </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>V5-bilocal has Schmidt rank&gt;1 generically</t>
+          <t>E-1 factorizable Psi^AB = Psi^A x Psi^B &amp; the tensor-product structure</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -2083,17 +2166,22 @@
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>P-V5-Schmidt-Generic — derivability from V5 envelope alone is OPEN</t>
-        </is>
-      </c>
+      <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr"/>
+          <t>P-Bipartite-Mapping — 'definitional commitment, not a separate derivation'</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-28</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2101,12 +2189,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n">
-        <v>65</v>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>064</t>
+        </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Monogamy budget cap; measure saturates the budget</t>
+          <t>V5-bilocal has Schmidt rank&gt;1 generically</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2115,17 +2205,18 @@
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>P-V5-Budget, P-Measure-Saturation</t>
-        </is>
-      </c>
+      <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr"/>
+          <t>P-V5-Schmidt-Generic — derivability from V5 envelope alone is OPEN</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2133,12 +2224,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B47" s="2" t="n">
-        <v>69</v>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>065</t>
+        </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>ED sits at Tsirelson; PR-boxes excluded</t>
+          <t>Monogamy budget cap; measure saturates the budget</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2147,17 +2240,18 @@
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>P-V5-Hilbert-Constraint</t>
-        </is>
-      </c>
+      <c r="F47" s="2" t="inlineStr"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr"/>
+          <t>P-V5-Budget, P-Measure-Saturation</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2165,35 +2259,34 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B48" s="2" t="n">
-        <v>63</v>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>069</t>
+        </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>E-2 non-factorizability is IRREDUCIBLE</t>
+          <t>ED sits at Tsirelson; PR-boxes excluded</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Asserted</t>
+          <t>Postulated</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>A-&gt;assertion — 'does not supply an explicit irreducibility proof' (round-5: was D, now A)</t>
-        </is>
-      </c>
+      <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>current — the arc's load-bearing soft spot</t>
+          <t>P-V5-Hilbert-Constraint</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>yes 2026-07-28</t>
-        </is>
-      </c>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2201,12 +2294,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B49" s="2" t="n">
-        <v>71</v>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>063</t>
+        </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>ER=EPR-class echo</t>
+          <t>E-2 non-factorizability is IRREDUCIBLE</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2215,17 +2310,22 @@
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>A-&gt;position — 'does NOT derive ER=EPR constructively'; rests on P-V5-Shared-EntanglementGravity</t>
-        </is>
-      </c>
+      <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr"/>
+          <t>A-&gt;assertion — 'does not supply an explicit irreducibility proof' (round-5: was D, now A)</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>current — the arc's load-bearing soft spot</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>yes 2026-07-28</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2233,12 +2333,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B50" s="2" t="n">
-        <v>72</v>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>071</t>
+        </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Entanglement = unresolved individuation regime (not action-at-a-distance)</t>
+          <t>ER=EPR-class echo</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -2247,17 +2349,18 @@
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>A-&gt;position — interpretive framing; does not modify QM predictions</t>
-        </is>
-      </c>
+      <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>current</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr"/>
+          <t>A-&gt;position — 'does NOT derive ER=EPR constructively'; rests on P-V5-Shared-EntanglementGravity</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2265,31 +2368,34 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B51" s="2" t="n">
-        <v>70</v>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>072</t>
+        </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Bipartite architecture as one phenomenon</t>
+          <t>Entanglement = unresolved individuation regime (not action-at-a-distance)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Synthesis</t>
+          <t>Asserted</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>A-&gt;position — 'does not override or strengthen constituent verdicts'</t>
-        </is>
-      </c>
+      <c r="F51" s="2" t="inlineStr"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>current (consolidation)</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr"/>
+          <t>A-&gt;position — interpretive framing; does not modify QM predictions</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2297,27 +2403,34 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B52" s="2" t="n">
-        <v>67</v>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>070</t>
+        </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>von Neumann E-6 (duplicate)</t>
+          <t>Bipartite architecture as one phenomenon</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Superseded</t>
+          <t>Synthesis</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>SUPERSEDED by 068 (merged 2026-07-05); kept for provenance</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr"/>
+          <t>A-&gt;position — 'does not override or strengthen constituent verdicts'</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>current (consolidation)</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2325,31 +2438,30 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B53" s="2" t="n">
-        <v>64</v>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>067</t>
+        </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>derivability of P-V5-Schmidt-Generic</t>
+          <t>von Neumann E-6 (duplicate)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Superseded</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr"/>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>SUPERSEDED by 068 (merged 2026-07-05); kept for provenance</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2357,12 +2469,14 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B54" s="2" t="n">
-        <v>68</v>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>064</t>
+        </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>O-vN-1: derive P-Additivity from P04 (quantitative)</t>
+          <t>derivability of P-V5-Schmidt-Generic</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2371,17 +2485,18 @@
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2389,34 +2504,72 @@
           <t>Entanglement</t>
         </is>
       </c>
-      <c r="B55" s="2" t="n">
-        <v>68</v>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>068</t>
+        </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
+          <t>O-vN-1: derive P-Additivity from P04 (quantitative)</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Entanglement</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>068</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
           <t>O-vN-2: derive P-Maximality from P11</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr"/>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>OPEN — structurally blocked; ED has no substrate-level temperature</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H55"/>
+  <autoFilter ref="A1:I56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add a 'Tier Key' sheet to the master (ranking + definitions)
Second sheet in ED_TieredClaims_Master.xlsx: Rank | Tier | Kind | Definition
| Rows, one row per tier (19), in the same rank order the Claims sheet sorts
by. Kind groups them Claim / Input / Meta. Rows = count per tier (sums to
401, a self-check vs the Claims sheet). Tier order + definitions live at
module level in the builder so the sort and the key can't drift.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ED_TieredClaims_Master.xlsx
+++ b/ED_TieredClaims_Master.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Claims" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tier Key" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Claims'!$A$1:$I$402</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tier Key'!$A$1:$E$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -15882,4 +15884,490 @@
   <autoFilter ref="A1:I402"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="108" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Standing</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>A settled result from another ED arc, cited here and built on — not re-derived in this folder.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Forced/proven from the 13 primitives (+ standard math) with NO paper-specific postulate — the strongest claim tier (theorems; M1).</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>D-via-I / Form-forced</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>The FORM is derived by composing inherited/standard pieces (derived-via-inherited); the form is forced, the numbers inherited.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Grounded</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Structural / conditional / account-tier: form-forced GIVEN a stated input or a declared paper-specific postulate (M2/M3).</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>A canonical DEFINITION or catalogue (a kernel, the verdict grammar, an audit) — scaffolding, not a claim to be proven.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Measured</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>A simulation / build-and-run / probe result on the certified substrate (or a faithful model of it).</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Inherited / Consilience</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Reproduces a known result/sequence framed THROUGH the substrate — supporting consilience, NOT a novel prediction.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Native / V5-conditional</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Mechanism is native but rests on V5, a faithful structural addition not shown primitive-forced.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Selected/Inherited</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A value taken from measurement, or a principled selection among a theorem's allowed options — not substrate-derived.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Constant</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>A fundamental constant, by when it enters: event-scale (units, present at the first events) / derived-combination / inherited-late.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Primitive</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>One of the 13 postulated axioms (P01-P13) — the corpus's single 'conditional on'; postulated, not derived, not claimed minimal.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Postulated</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Rests on a named paper-specific postulate (a declared commitment BEYOND the 13 primitives).</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Asserted</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>An A-&gt;position / A-&gt;assertion: stated in the paper's own audit as a position, NOT proven (the weakest claim tier).</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Prediction</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>A falsifiable, experiment-facing bet — carries a kill-condition (see the Falsifier / Kill-Cond column).</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Identification</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>A structural mapping onto an existing EXTERNAL framework (e.g. Penrose CCC, Jacobson's equation of state).</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Wall</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Claim</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>A proven or honestly-checked LIMIT — the order or result ED does NOT reach (a load-bearing 'no').</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Synthesis</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>An arc consolidation / overview / organizing lens; composes standing results, adds no new derivation.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Superseded</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Retracted / withdrawn / superseded by a later corpus result (kept for provenance).</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>A declared OPEN / unclosed item — a named gap or frontier.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E20"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add an 'Untunability' sheet: domains reproduced / free inputs, both framings
Third sheet in the master, computed from the Claims data:
- Ingredients: 12 domains, 172 reproduced-structure claims (by tier), 23
  predictions, 13 shared primitives, ~4 shared inherited scales, the inherited
  matter sector, ~15 live paper-specific postulates (24 total -6 Foundations
  meta-rows -3 discharged/definitional).
- Framing 1 (domains per shared primitive: 12/13 ~ 0.92) and Framing 2 (fixed
  denominator, growing numerator) side by side, each with its interpretation.
- Bottom caveat: why results/rows (172/88) is meaningless -- counts DOMAINS and
  SHARED inputs, assumptions stated in-cell so it reads as an argument, not a
  headline number.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ED_TieredClaims_Master.xlsx
+++ b/ED_TieredClaims_Master.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Claims" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Tier Key" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Untunability" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Claims'!$A$1:$I$402</definedName>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +39,28 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -79,12 +102,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -16370,4 +16414,221 @@
   <autoFilter ref="A1:E20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="72" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Untunability — the figure of merit: domains reproduced ÷ free inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>A proxy for “could you have tuned it?” — the answer is NO when the denominator is small AND shared. This counts DOMAINS (folders) and SHARED inputs, not claim-rows (see the caveat at the bottom).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Ingredients (computed from the Claims sheet)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Domains reproduced (independent physics folders)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>each with its standard structure form-reproduced; grows as you add sectors</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Reproduced-structure claims across them</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Standing 7 / Derived 50 / D-via-I 13 / Grounded 82 / Measured 12 / Inherited 4 / Native 1 / Identification 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Forward predictions (separate; NOT reproductions)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>the falsifiable bets — not part of the reproduction count</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>— Shared axioms: the 13 primitives (P01–P13)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ONE set, shared across ALL domains — not 13-per-domain. The load-bearing fact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>— Shared inherited scales</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>c, ħ, ℓ_P (= units, all 1) + H₀ (sets BOTH a₀ and Λ). G is derived; a₀/Λ are H₀-derived — not free knobs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>— Matter-sector values (inherited, as the SM's ~20)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>masses, couplings, α — openly inherited, not ED-fixed (same status as the Standard Model)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>— Live paper-specific postulates</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>~15</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>of 24 Postulated rows: −6 Foundations meta-rows (about the axiom system), −3 discharged/definitional (P14→QuadraticStrain, P-GW-Saddle=naming, P-NonAbelian-Analogy→MS-II). The only per-domain knobs; some still shared (V5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>FRAMING 1 — domains per shared primitive</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>FRAMING 2 — fixed denominator, growing numerator</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>12 domains ÷ 13 shared axioms  ≈  0.92 domains / primitive</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>denominator = 13 (fixed)   ·   numerator = 12 (and growing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="150" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>But this UNDERSELLS it: each of the 13 primitives feeds MANY domains, so they are reused, not spent per domain. The honest read is not “0.9” — it is that ~12 unrelated domains (gravity, the Born rule, viscoelastic relaxation, the dark sector…) come out of ONE 13-axiom structure. You cannot tune 13 shared primitives to independently hit that many unrelated fields by accident, because they all run through the SAME primitives.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Add a domain and the numerator rises; the denominator (13 primitives) does NOT. Contrast “a theory per domain” — GR + QM + a dark-matter particle + brute constants — where each new domain brings its OWN axioms AND its own inputs. ED adds domains at ~0 new-axiom cost. So the figure of merit is not a number to maximize; it is that the denominator refuses to grow while the numerator does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="78" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Why NOT results ÷ rows (172 / 88 ≈ 2 is meaningless): (1) numerator granularity is arbitrary — a folder is one domain but many rows (gravity 45, state-reduction 15); (2) the 41 Selected/Inherited rows are only ~5 DISTINCT values re-cited across folders (ħ, ℓ_P, c… counted once per folder is not a new knob); (3) the 24 Postulated rows include discharged and definitional-only ones. This sheet deliberately counts DOMAINS and SHARED inputs. Assumptions are stated in-cell so this reads as an argument, not a headline number.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="E14:G14"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="E15:G15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add a 'Postulate' discharged-flag column to the Postulated rows
New column on the Claims sheet, populated only for Tier=Postulated (blank
elsewhere): live / discharged / definitional / meta.
  - live (15): substantive still-load-bearing per-domain postulates (the real knobs)
  - discharged (2): P14 -> QuadraticStrain; P-NonAbelian-Analogy -> MS-II §2 derivation
  - definitional (1): P-GW-SaddleReconfiguration (naming convention only)
  - meta (6): Foundations rows about the axiom system, not per-domain knobs

The Untunability sheet's 'live paper-specific postulates' now reads this flag
(exact 15, not a hardcoded subtraction) and breaks the 24 down by category.
Classifier is in the builder so it stays reproducible on rebuild.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ED_TieredClaims_Master.xlsx
+++ b/ED_TieredClaims_Master.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Untunability" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Claims'!$A$1:$I$402</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Claims'!$A$1:$J$402</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tier Key'!$A$1:$E$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I402"/>
+  <dimension ref="A1:J402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -508,6 +508,7 @@
     <col width="44" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -556,6 +557,11 @@
           <t>SpotChecked</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Postulate</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -599,6 +605,7 @@
           <t>yes 2026-07-29 (read in full before import)</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -642,6 +649,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -681,6 +689,7 @@
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -720,6 +729,7 @@
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -763,6 +773,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -802,6 +813,7 @@
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -841,6 +853,7 @@
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -880,6 +893,7 @@
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -919,6 +933,7 @@
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -958,6 +973,7 @@
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -997,6 +1013,7 @@
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1036,6 +1053,7 @@
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1075,6 +1093,7 @@
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1114,6 +1133,7 @@
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1157,6 +1177,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1196,6 +1217,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1231,6 +1253,7 @@
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1266,6 +1289,7 @@
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1301,6 +1325,7 @@
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1336,6 +1361,7 @@
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1371,6 +1397,7 @@
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1406,6 +1433,7 @@
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1441,6 +1469,7 @@
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1480,6 +1509,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1523,6 +1553,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1558,6 +1589,7 @@
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1593,6 +1625,7 @@
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1628,6 +1661,7 @@
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1663,6 +1697,7 @@
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1698,6 +1733,7 @@
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1733,6 +1769,7 @@
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1772,6 +1809,7 @@
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1807,6 +1845,7 @@
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1842,6 +1881,7 @@
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1881,6 +1921,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1916,6 +1957,7 @@
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1951,6 +1993,7 @@
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1986,6 +2029,7 @@
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2025,6 +2069,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2068,6 +2113,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2103,6 +2149,7 @@
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2138,6 +2185,7 @@
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2177,6 +2225,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2216,6 +2265,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2251,6 +2301,7 @@
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2286,6 +2337,7 @@
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2321,6 +2373,7 @@
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2356,6 +2409,7 @@
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2391,6 +2445,7 @@
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2434,6 +2489,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2473,6 +2529,7 @@
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2512,6 +2569,7 @@
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2555,6 +2613,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2598,6 +2657,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2637,6 +2697,7 @@
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2680,6 +2741,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2719,6 +2781,7 @@
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2758,6 +2821,7 @@
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2797,6 +2861,7 @@
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2836,6 +2901,7 @@
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2871,6 +2937,7 @@
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2906,6 +2973,7 @@
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2941,6 +3009,7 @@
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2976,6 +3045,7 @@
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3015,6 +3085,11 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3054,6 +3129,7 @@
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3093,6 +3169,7 @@
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -3132,6 +3209,7 @@
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -3171,6 +3249,7 @@
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3206,6 +3285,7 @@
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3241,6 +3321,7 @@
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3280,6 +3361,7 @@
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr"/>
+      <c r="J73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3319,6 +3401,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3354,6 +3437,7 @@
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3389,6 +3473,7 @@
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3424,6 +3509,7 @@
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3459,6 +3545,7 @@
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3494,6 +3581,7 @@
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3529,6 +3617,7 @@
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3564,6 +3653,7 @@
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3603,6 +3693,7 @@
           <t>yes 2026-07-29 (read in full)</t>
         </is>
       </c>
+      <c r="J82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3646,6 +3737,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3689,6 +3781,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3732,6 +3825,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3775,6 +3869,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -3822,6 +3917,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3869,6 +3965,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3912,6 +4009,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3951,6 +4049,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3990,6 +4089,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -4029,6 +4129,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -4068,6 +4169,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4111,6 +4213,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -4150,6 +4253,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -4189,6 +4293,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -4228,6 +4333,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -4271,6 +4377,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4314,6 +4421,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -4357,6 +4465,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4396,6 +4505,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4435,6 +4545,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -4478,6 +4589,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -4517,6 +4629,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -4556,6 +4669,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J105" s="2" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -4595,6 +4709,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -4634,6 +4749,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J107" s="2" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4677,6 +4793,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -4716,6 +4833,7 @@
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr"/>
+      <c r="J109" s="2" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4759,6 +4877,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4798,6 +4917,7 @@
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr"/>
+      <c r="J111" s="2" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -4837,6 +4957,7 @@
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -4880,6 +5001,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J113" s="2" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -4919,6 +5041,7 @@
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr"/>
+      <c r="J114" s="2" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -4958,6 +5081,7 @@
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr"/>
+      <c r="J115" s="2" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5001,6 +5125,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -5036,6 +5161,7 @@
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr"/>
+      <c r="J117" s="2" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -5075,6 +5201,7 @@
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr"/>
+      <c r="J118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -5114,6 +5241,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J119" s="2" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -5149,6 +5277,7 @@
         </is>
       </c>
       <c r="I120" s="2" t="inlineStr"/>
+      <c r="J120" s="2" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -5184,6 +5313,7 @@
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr"/>
+      <c r="J121" s="2" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -5219,6 +5349,11 @@
         </is>
       </c>
       <c r="I122" s="2" t="inlineStr"/>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
+          <t>definitional</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -5254,6 +5389,7 @@
         </is>
       </c>
       <c r="I123" s="2" t="inlineStr"/>
+      <c r="J123" s="2" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -5293,6 +5429,7 @@
         </is>
       </c>
       <c r="I124" s="2" t="inlineStr"/>
+      <c r="J124" s="2" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -5328,6 +5465,7 @@
         </is>
       </c>
       <c r="I125" s="2" t="inlineStr"/>
+      <c r="J125" s="2" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -5363,6 +5501,7 @@
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr"/>
+      <c r="J126" s="2" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -5398,6 +5537,7 @@
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr"/>
+      <c r="J127" s="2" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -5433,6 +5573,7 @@
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr"/>
+      <c r="J128" s="2" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -5472,6 +5613,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J129" s="2" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -5511,6 +5653,7 @@
         </is>
       </c>
       <c r="I130" s="2" t="inlineStr"/>
+      <c r="J130" s="2" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -5550,6 +5693,7 @@
         </is>
       </c>
       <c r="I131" s="2" t="inlineStr"/>
+      <c r="J131" s="2" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -5593,6 +5737,7 @@
           <t>yes 2026-07-28</t>
         </is>
       </c>
+      <c r="J132" s="2" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -5632,6 +5777,7 @@
         </is>
       </c>
       <c r="I133" s="2" t="inlineStr"/>
+      <c r="J133" s="2" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -5671,6 +5817,7 @@
           <t>yes 2026-07-28</t>
         </is>
       </c>
+      <c r="J134" s="2" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -5706,6 +5853,7 @@
         </is>
       </c>
       <c r="I135" s="2" t="inlineStr"/>
+      <c r="J135" s="2" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -5741,6 +5889,7 @@
         </is>
       </c>
       <c r="I136" s="2" t="inlineStr"/>
+      <c r="J136" s="2" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -5776,6 +5925,7 @@
         </is>
       </c>
       <c r="I137" s="2" t="inlineStr"/>
+      <c r="J137" s="2" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -5819,6 +5969,7 @@
           <t>yes 2026-07-28</t>
         </is>
       </c>
+      <c r="J138" s="2" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -5858,6 +6009,11 @@
           <t>yes 2026-07-28</t>
         </is>
       </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -5893,6 +6049,11 @@
         </is>
       </c>
       <c r="I140" s="2" t="inlineStr"/>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -5928,6 +6089,11 @@
         </is>
       </c>
       <c r="I141" s="2" t="inlineStr"/>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -5963,6 +6129,11 @@
         </is>
       </c>
       <c r="I142" s="2" t="inlineStr"/>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -6002,6 +6173,7 @@
           <t>yes 2026-07-28</t>
         </is>
       </c>
+      <c r="J143" s="2" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -6037,6 +6209,7 @@
         </is>
       </c>
       <c r="I144" s="2" t="inlineStr"/>
+      <c r="J144" s="2" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -6072,6 +6245,7 @@
         </is>
       </c>
       <c r="I145" s="2" t="inlineStr"/>
+      <c r="J145" s="2" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -6107,6 +6281,7 @@
         </is>
       </c>
       <c r="I146" s="2" t="inlineStr"/>
+      <c r="J146" s="2" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -6138,6 +6313,7 @@
         </is>
       </c>
       <c r="I147" s="2" t="inlineStr"/>
+      <c r="J147" s="2" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -6173,6 +6349,7 @@
         </is>
       </c>
       <c r="I148" s="2" t="inlineStr"/>
+      <c r="J148" s="2" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -6208,6 +6385,7 @@
         </is>
       </c>
       <c r="I149" s="2" t="inlineStr"/>
+      <c r="J149" s="2" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -6243,6 +6421,7 @@
         </is>
       </c>
       <c r="I150" s="2" t="inlineStr"/>
+      <c r="J150" s="2" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -6282,6 +6461,7 @@
         </is>
       </c>
       <c r="I151" s="2" t="inlineStr"/>
+      <c r="J151" s="2" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -6325,6 +6505,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J152" s="2" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -6364,6 +6545,7 @@
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr"/>
+      <c r="J153" s="2" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -6403,6 +6585,7 @@
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr"/>
+      <c r="J154" s="2" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -6438,6 +6621,7 @@
         </is>
       </c>
       <c r="I155" s="2" t="inlineStr"/>
+      <c r="J155" s="2" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -6477,6 +6661,7 @@
         </is>
       </c>
       <c r="I156" s="2" t="inlineStr"/>
+      <c r="J156" s="2" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -6520,6 +6705,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J157" s="2" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -6563,6 +6749,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J158" s="2" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -6598,6 +6785,7 @@
         </is>
       </c>
       <c r="I159" s="2" t="inlineStr"/>
+      <c r="J159" s="2" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -6633,6 +6821,7 @@
         </is>
       </c>
       <c r="I160" s="2" t="inlineStr"/>
+      <c r="J160" s="2" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -6668,6 +6857,7 @@
         </is>
       </c>
       <c r="I161" s="2" t="inlineStr"/>
+      <c r="J161" s="2" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -6703,6 +6893,7 @@
         </is>
       </c>
       <c r="I162" s="2" t="inlineStr"/>
+      <c r="J162" s="2" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -6742,6 +6933,11 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J163" s="2" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -6777,6 +6973,11 @@
         </is>
       </c>
       <c r="I164" s="2" t="inlineStr"/>
+      <c r="J164" s="2" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -6812,6 +7013,11 @@
         </is>
       </c>
       <c r="I165" s="2" t="inlineStr"/>
+      <c r="J165" s="2" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -6847,6 +7053,11 @@
         </is>
       </c>
       <c r="I166" s="2" t="inlineStr"/>
+      <c r="J166" s="2" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -6882,6 +7093,11 @@
         </is>
       </c>
       <c r="I167" s="2" t="inlineStr"/>
+      <c r="J167" s="2" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -6921,6 +7137,11 @@
         </is>
       </c>
       <c r="I168" s="2" t="inlineStr"/>
+      <c r="J168" s="2" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -6960,6 +7181,7 @@
         </is>
       </c>
       <c r="I169" s="2" t="inlineStr"/>
+      <c r="J169" s="2" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -6999,6 +7221,7 @@
         </is>
       </c>
       <c r="I170" s="2" t="inlineStr"/>
+      <c r="J170" s="2" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -7038,6 +7261,7 @@
         </is>
       </c>
       <c r="I171" s="2" t="inlineStr"/>
+      <c r="J171" s="2" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -7077,6 +7301,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J172" s="2" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -7112,6 +7337,7 @@
         </is>
       </c>
       <c r="I173" s="2" t="inlineStr"/>
+      <c r="J173" s="2" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -7147,6 +7373,7 @@
         </is>
       </c>
       <c r="I174" s="2" t="inlineStr"/>
+      <c r="J174" s="2" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -7182,6 +7409,7 @@
         </is>
       </c>
       <c r="I175" s="2" t="inlineStr"/>
+      <c r="J175" s="2" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -7217,6 +7445,7 @@
         </is>
       </c>
       <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -7256,6 +7485,7 @@
         </is>
       </c>
       <c r="I177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -7295,6 +7525,7 @@
         </is>
       </c>
       <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -7334,6 +7565,7 @@
         </is>
       </c>
       <c r="I179" s="2" t="inlineStr"/>
+      <c r="J179" s="2" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -7373,6 +7605,7 @@
         </is>
       </c>
       <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -7412,6 +7645,7 @@
         </is>
       </c>
       <c r="I181" s="2" t="inlineStr"/>
+      <c r="J181" s="2" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -7455,6 +7689,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J182" s="2" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -7494,6 +7729,7 @@
         </is>
       </c>
       <c r="I183" s="2" t="inlineStr"/>
+      <c r="J183" s="2" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -7533,6 +7769,7 @@
         </is>
       </c>
       <c r="I184" s="2" t="inlineStr"/>
+      <c r="J184" s="2" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -7572,6 +7809,7 @@
         </is>
       </c>
       <c r="I185" s="2" t="inlineStr"/>
+      <c r="J185" s="2" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -7611,6 +7849,7 @@
         </is>
       </c>
       <c r="I186" s="2" t="inlineStr"/>
+      <c r="J186" s="2" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -7650,6 +7889,7 @@
         </is>
       </c>
       <c r="I187" s="2" t="inlineStr"/>
+      <c r="J187" s="2" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -7689,6 +7929,7 @@
         </is>
       </c>
       <c r="I188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -7728,6 +7969,7 @@
         </is>
       </c>
       <c r="I189" s="2" t="inlineStr"/>
+      <c r="J189" s="2" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -7771,6 +8013,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J190" s="2" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -7810,6 +8053,7 @@
         </is>
       </c>
       <c r="I191" s="2" t="inlineStr"/>
+      <c r="J191" s="2" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -7853,6 +8097,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J192" s="2" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -7892,6 +8137,7 @@
         </is>
       </c>
       <c r="I193" s="2" t="inlineStr"/>
+      <c r="J193" s="2" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -7931,6 +8177,7 @@
         </is>
       </c>
       <c r="I194" s="2" t="inlineStr"/>
+      <c r="J194" s="2" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -7974,6 +8221,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J195" s="2" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -8017,6 +8265,7 @@
           <t>yes 2026-07-29 (corroborated via 030/QuadraticStrain checks)</t>
         </is>
       </c>
+      <c r="J196" s="2" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -8056,6 +8305,7 @@
         </is>
       </c>
       <c r="I197" s="2" t="inlineStr"/>
+      <c r="J197" s="2" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -8095,6 +8345,7 @@
         </is>
       </c>
       <c r="I198" s="2" t="inlineStr"/>
+      <c r="J198" s="2" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -8134,6 +8385,7 @@
         </is>
       </c>
       <c r="I199" s="2" t="inlineStr"/>
+      <c r="J199" s="2" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -8173,6 +8425,7 @@
         </is>
       </c>
       <c r="I200" s="2" t="inlineStr"/>
+      <c r="J200" s="2" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -8212,6 +8465,7 @@
         </is>
       </c>
       <c r="I201" s="2" t="inlineStr"/>
+      <c r="J201" s="2" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -8251,6 +8505,7 @@
         </is>
       </c>
       <c r="I202" s="2" t="inlineStr"/>
+      <c r="J202" s="2" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -8290,6 +8545,7 @@
         </is>
       </c>
       <c r="I203" s="2" t="inlineStr"/>
+      <c r="J203" s="2" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -8329,6 +8585,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J204" s="2" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -8368,6 +8625,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J205" s="2" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -8403,6 +8661,7 @@
         </is>
       </c>
       <c r="I206" s="2" t="inlineStr"/>
+      <c r="J206" s="2" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -8438,6 +8697,11 @@
         </is>
       </c>
       <c r="I207" s="2" t="inlineStr"/>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t>discharged</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -8473,6 +8737,11 @@
         </is>
       </c>
       <c r="I208" s="2" t="inlineStr"/>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -8508,6 +8777,11 @@
         </is>
       </c>
       <c r="I209" s="2" t="inlineStr"/>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -8551,6 +8825,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J210" s="2" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -8594,6 +8869,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J211" s="2" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -8633,6 +8909,7 @@
         </is>
       </c>
       <c r="I212" s="2" t="inlineStr"/>
+      <c r="J212" s="2" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -8672,6 +8949,7 @@
         </is>
       </c>
       <c r="I213" s="2" t="inlineStr"/>
+      <c r="J213" s="2" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -8715,6 +8993,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J214" s="2" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -8754,6 +9033,7 @@
         </is>
       </c>
       <c r="I215" s="2" t="inlineStr"/>
+      <c r="J215" s="2" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -8789,6 +9069,7 @@
         </is>
       </c>
       <c r="I216" s="2" t="inlineStr"/>
+      <c r="J216" s="2" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -8828,6 +9109,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J217" s="2" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -8863,6 +9145,7 @@
         </is>
       </c>
       <c r="I218" s="2" t="inlineStr"/>
+      <c r="J218" s="2" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -8898,6 +9181,7 @@
         </is>
       </c>
       <c r="I219" s="2" t="inlineStr"/>
+      <c r="J219" s="2" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -8933,6 +9217,7 @@
         </is>
       </c>
       <c r="I220" s="2" t="inlineStr"/>
+      <c r="J220" s="2" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -8972,6 +9257,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J221" s="2" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -9011,6 +9297,7 @@
         </is>
       </c>
       <c r="I222" s="2" t="inlineStr"/>
+      <c r="J222" s="2" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -9050,6 +9337,7 @@
         </is>
       </c>
       <c r="I223" s="2" t="inlineStr"/>
+      <c r="J223" s="2" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -9089,6 +9377,7 @@
         </is>
       </c>
       <c r="I224" s="2" t="inlineStr"/>
+      <c r="J224" s="2" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -9128,6 +9417,7 @@
         </is>
       </c>
       <c r="I225" s="2" t="inlineStr"/>
+      <c r="J225" s="2" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -9167,6 +9457,7 @@
         </is>
       </c>
       <c r="I226" s="2" t="inlineStr"/>
+      <c r="J226" s="2" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -9206,6 +9497,7 @@
         </is>
       </c>
       <c r="I227" s="2" t="inlineStr"/>
+      <c r="J227" s="2" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -9241,6 +9533,7 @@
         </is>
       </c>
       <c r="I228" s="2" t="inlineStr"/>
+      <c r="J228" s="2" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -9280,6 +9573,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J229" s="2" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -9315,6 +9609,7 @@
         </is>
       </c>
       <c r="I230" s="2" t="inlineStr"/>
+      <c r="J230" s="2" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -9350,6 +9645,7 @@
         </is>
       </c>
       <c r="I231" s="2" t="inlineStr"/>
+      <c r="J231" s="2" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -9385,6 +9681,7 @@
         </is>
       </c>
       <c r="I232" s="2" t="inlineStr"/>
+      <c r="J232" s="2" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -9420,6 +9717,7 @@
         </is>
       </c>
       <c r="I233" s="2" t="inlineStr"/>
+      <c r="J233" s="2" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -9459,6 +9757,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J234" s="2" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -9494,6 +9793,7 @@
         </is>
       </c>
       <c r="I235" s="2" t="inlineStr"/>
+      <c r="J235" s="2" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -9529,6 +9829,7 @@
         </is>
       </c>
       <c r="I236" s="2" t="inlineStr"/>
+      <c r="J236" s="2" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -9564,6 +9865,7 @@
         </is>
       </c>
       <c r="I237" s="2" t="inlineStr"/>
+      <c r="J237" s="2" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -9599,6 +9901,7 @@
         </is>
       </c>
       <c r="I238" s="2" t="inlineStr"/>
+      <c r="J238" s="2" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -9638,6 +9941,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J239" s="2" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -9673,6 +9977,7 @@
         </is>
       </c>
       <c r="I240" s="2" t="inlineStr"/>
+      <c r="J240" s="2" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -9712,6 +10017,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J241" s="2" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -9751,6 +10057,7 @@
         </is>
       </c>
       <c r="I242" s="2" t="inlineStr"/>
+      <c r="J242" s="2" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -9790,6 +10097,7 @@
         </is>
       </c>
       <c r="I243" s="2" t="inlineStr"/>
+      <c r="J243" s="2" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -9833,6 +10141,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J244" s="2" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -9868,6 +10177,7 @@
         </is>
       </c>
       <c r="I245" s="2" t="inlineStr"/>
+      <c r="J245" s="2" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
@@ -9907,6 +10217,7 @@
         </is>
       </c>
       <c r="I246" s="2" t="inlineStr"/>
+      <c r="J246" s="2" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
@@ -9946,6 +10257,7 @@
         </is>
       </c>
       <c r="I247" s="2" t="inlineStr"/>
+      <c r="J247" s="2" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
@@ -9989,6 +10301,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J248" s="2" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
@@ -10028,6 +10341,7 @@
         </is>
       </c>
       <c r="I249" s="2" t="inlineStr"/>
+      <c r="J249" s="2" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
@@ -10067,6 +10381,7 @@
         </is>
       </c>
       <c r="I250" s="2" t="inlineStr"/>
+      <c r="J250" s="2" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
@@ -10106,6 +10421,7 @@
         </is>
       </c>
       <c r="I251" s="2" t="inlineStr"/>
+      <c r="J251" s="2" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -10145,6 +10461,7 @@
         </is>
       </c>
       <c r="I252" s="2" t="inlineStr"/>
+      <c r="J252" s="2" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" s="2" t="inlineStr">
@@ -10180,6 +10497,7 @@
         </is>
       </c>
       <c r="I253" s="2" t="inlineStr"/>
+      <c r="J253" s="2" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -10219,6 +10537,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J254" s="2" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">
@@ -10254,6 +10573,7 @@
         </is>
       </c>
       <c r="I255" s="2" t="inlineStr"/>
+      <c r="J255" s="2" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="2" t="inlineStr">
@@ -10297,6 +10617,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J256" s="2" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
@@ -10332,6 +10653,7 @@
         </is>
       </c>
       <c r="I257" s="2" t="inlineStr"/>
+      <c r="J257" s="2" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" s="2" t="inlineStr">
@@ -10375,6 +10697,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J258" s="2" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
@@ -10410,6 +10733,7 @@
         </is>
       </c>
       <c r="I259" s="2" t="inlineStr"/>
+      <c r="J259" s="2" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
@@ -10445,6 +10769,7 @@
         </is>
       </c>
       <c r="I260" s="2" t="inlineStr"/>
+      <c r="J260" s="2" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
@@ -10480,6 +10805,7 @@
         </is>
       </c>
       <c r="I261" s="2" t="inlineStr"/>
+      <c r="J261" s="2" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
@@ -10515,6 +10841,7 @@
         </is>
       </c>
       <c r="I262" s="2" t="inlineStr"/>
+      <c r="J262" s="2" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
@@ -10550,6 +10877,7 @@
         </is>
       </c>
       <c r="I263" s="2" t="inlineStr"/>
+      <c r="J263" s="2" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
@@ -10585,6 +10913,7 @@
         </is>
       </c>
       <c r="I264" s="2" t="inlineStr"/>
+      <c r="J264" s="2" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
@@ -10620,6 +10949,7 @@
         </is>
       </c>
       <c r="I265" s="2" t="inlineStr"/>
+      <c r="J265" s="2" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
@@ -10659,6 +10989,7 @@
         </is>
       </c>
       <c r="I266" s="2" t="inlineStr"/>
+      <c r="J266" s="2" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" s="2" t="inlineStr">
@@ -10694,6 +11025,7 @@
         </is>
       </c>
       <c r="I267" s="2" t="inlineStr"/>
+      <c r="J267" s="2" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="2" t="inlineStr">
@@ -10733,6 +11065,7 @@
         </is>
       </c>
       <c r="I268" s="2" t="inlineStr"/>
+      <c r="J268" s="2" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
@@ -10776,6 +11109,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J269" s="2" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
@@ -10815,6 +11149,7 @@
         </is>
       </c>
       <c r="I270" s="2" t="inlineStr"/>
+      <c r="J270" s="2" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
@@ -10854,6 +11189,7 @@
         </is>
       </c>
       <c r="I271" s="2" t="inlineStr"/>
+      <c r="J271" s="2" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
@@ -10897,6 +11233,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J272" s="2" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -10936,6 +11273,7 @@
         </is>
       </c>
       <c r="I273" s="2" t="inlineStr"/>
+      <c r="J273" s="2" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
@@ -10975,6 +11313,7 @@
         </is>
       </c>
       <c r="I274" s="2" t="inlineStr"/>
+      <c r="J274" s="2" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
@@ -11018,6 +11357,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J275" s="2" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
@@ -11057,6 +11397,7 @@
         </is>
       </c>
       <c r="I276" s="2" t="inlineStr"/>
+      <c r="J276" s="2" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
@@ -11096,6 +11437,7 @@
         </is>
       </c>
       <c r="I277" s="2" t="inlineStr"/>
+      <c r="J277" s="2" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
@@ -11135,6 +11477,7 @@
         </is>
       </c>
       <c r="I278" s="2" t="inlineStr"/>
+      <c r="J278" s="2" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
@@ -11178,6 +11521,7 @@
         </is>
       </c>
       <c r="I279" s="2" t="inlineStr"/>
+      <c r="J279" s="2" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
@@ -11221,6 +11565,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J280" s="2" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
@@ -11264,6 +11609,7 @@
         </is>
       </c>
       <c r="I281" s="2" t="inlineStr"/>
+      <c r="J281" s="2" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
@@ -11303,6 +11649,7 @@
         </is>
       </c>
       <c r="I282" s="2" t="inlineStr"/>
+      <c r="J282" s="2" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" s="2" t="inlineStr">
@@ -11338,6 +11685,7 @@
         </is>
       </c>
       <c r="I283" s="2" t="inlineStr"/>
+      <c r="J283" s="2" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" s="2" t="inlineStr">
@@ -11377,6 +11725,7 @@
         </is>
       </c>
       <c r="I284" s="2" t="inlineStr"/>
+      <c r="J284" s="2" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" s="2" t="inlineStr">
@@ -11416,6 +11765,7 @@
         </is>
       </c>
       <c r="I285" s="2" t="inlineStr"/>
+      <c r="J285" s="2" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
@@ -11451,6 +11801,7 @@
         </is>
       </c>
       <c r="I286" s="2" t="inlineStr"/>
+      <c r="J286" s="2" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" s="2" t="inlineStr">
@@ -11486,6 +11837,7 @@
         </is>
       </c>
       <c r="I287" s="2" t="inlineStr"/>
+      <c r="J287" s="2" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
@@ -11521,6 +11873,7 @@
         </is>
       </c>
       <c r="I288" s="2" t="inlineStr"/>
+      <c r="J288" s="2" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
@@ -11556,6 +11909,11 @@
         </is>
       </c>
       <c r="I289" s="2" t="inlineStr"/>
+      <c r="J289" s="2" t="inlineStr">
+        <is>
+          <t>discharged</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
@@ -11591,6 +11949,11 @@
         </is>
       </c>
       <c r="I290" s="2" t="inlineStr"/>
+      <c r="J290" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
@@ -11626,6 +11989,11 @@
         </is>
       </c>
       <c r="I291" s="2" t="inlineStr"/>
+      <c r="J291" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
@@ -11661,6 +12029,11 @@
         </is>
       </c>
       <c r="I292" s="2" t="inlineStr"/>
+      <c r="J292" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
@@ -11696,6 +12069,7 @@
         </is>
       </c>
       <c r="I293" s="2" t="inlineStr"/>
+      <c r="J293" s="2" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
@@ -11735,6 +12109,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J294" s="2" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
@@ -11774,6 +12149,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J295" s="2" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
@@ -11809,6 +12185,7 @@
         </is>
       </c>
       <c r="I296" s="2" t="inlineStr"/>
+      <c r="J296" s="2" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
@@ -11848,6 +12225,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J297" s="2" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
@@ -11883,6 +12261,7 @@
         </is>
       </c>
       <c r="I298" s="2" t="inlineStr"/>
+      <c r="J298" s="2" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
@@ -11918,6 +12297,7 @@
         </is>
       </c>
       <c r="I299" s="2" t="inlineStr"/>
+      <c r="J299" s="2" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
@@ -11961,6 +12341,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J300" s="2" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
@@ -12000,6 +12381,7 @@
         </is>
       </c>
       <c r="I301" s="2" t="inlineStr"/>
+      <c r="J301" s="2" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
@@ -12039,6 +12421,7 @@
         </is>
       </c>
       <c r="I302" s="2" t="inlineStr"/>
+      <c r="J302" s="2" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
@@ -12078,6 +12461,7 @@
         </is>
       </c>
       <c r="I303" s="2" t="inlineStr"/>
+      <c r="J303" s="2" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
@@ -12117,6 +12501,7 @@
         </is>
       </c>
       <c r="I304" s="2" t="inlineStr"/>
+      <c r="J304" s="2" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
@@ -12160,6 +12545,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J305" s="2" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
@@ -12199,6 +12585,7 @@
         </is>
       </c>
       <c r="I306" s="2" t="inlineStr"/>
+      <c r="J306" s="2" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
@@ -12242,6 +12629,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J307" s="2" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
@@ -12281,6 +12669,7 @@
         </is>
       </c>
       <c r="I308" s="2" t="inlineStr"/>
+      <c r="J308" s="2" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
@@ -12320,6 +12709,7 @@
         </is>
       </c>
       <c r="I309" s="2" t="inlineStr"/>
+      <c r="J309" s="2" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
@@ -12359,6 +12749,7 @@
         </is>
       </c>
       <c r="I310" s="2" t="inlineStr"/>
+      <c r="J310" s="2" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
@@ -12398,6 +12789,7 @@
         </is>
       </c>
       <c r="I311" s="2" t="inlineStr"/>
+      <c r="J311" s="2" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
@@ -12437,6 +12829,7 @@
         </is>
       </c>
       <c r="I312" s="2" t="inlineStr"/>
+      <c r="J312" s="2" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
@@ -12476,6 +12869,7 @@
         </is>
       </c>
       <c r="I313" s="2" t="inlineStr"/>
+      <c r="J313" s="2" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
@@ -12515,6 +12909,7 @@
         </is>
       </c>
       <c r="I314" s="2" t="inlineStr"/>
+      <c r="J314" s="2" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
@@ -12554,6 +12949,7 @@
         </is>
       </c>
       <c r="I315" s="2" t="inlineStr"/>
+      <c r="J315" s="2" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
@@ -12593,6 +12989,7 @@
         </is>
       </c>
       <c r="I316" s="2" t="inlineStr"/>
+      <c r="J316" s="2" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
@@ -12632,6 +13029,7 @@
         </is>
       </c>
       <c r="I317" s="2" t="inlineStr"/>
+      <c r="J317" s="2" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
@@ -12675,6 +13073,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J318" s="2" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
@@ -12718,6 +13117,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J319" s="2" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
@@ -12753,6 +13153,7 @@
         </is>
       </c>
       <c r="I320" s="2" t="inlineStr"/>
+      <c r="J320" s="2" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
@@ -12788,6 +13189,7 @@
         </is>
       </c>
       <c r="I321" s="2" t="inlineStr"/>
+      <c r="J321" s="2" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
@@ -12827,6 +13229,7 @@
         </is>
       </c>
       <c r="I322" s="2" t="inlineStr"/>
+      <c r="J322" s="2" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
@@ -12866,6 +13269,11 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J323" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
@@ -12901,6 +13309,11 @@
         </is>
       </c>
       <c r="I324" s="2" t="inlineStr"/>
+      <c r="J324" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
@@ -12936,6 +13349,7 @@
         </is>
       </c>
       <c r="I325" s="2" t="inlineStr"/>
+      <c r="J325" s="2" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
@@ -12975,6 +13389,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J326" s="2" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
@@ -13018,6 +13433,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J327" s="2" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
@@ -13061,6 +13477,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J328" s="2" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
@@ -13108,6 +13525,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J329" s="2" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
@@ -13151,6 +13569,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J330" s="2" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
@@ -13194,6 +13613,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J331" s="2" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
@@ -13233,6 +13653,7 @@
         </is>
       </c>
       <c r="I332" s="2" t="inlineStr"/>
+      <c r="J332" s="2" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
@@ -13272,6 +13693,7 @@
         </is>
       </c>
       <c r="I333" s="2" t="inlineStr"/>
+      <c r="J333" s="2" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
@@ -13311,6 +13733,7 @@
         </is>
       </c>
       <c r="I334" s="2" t="inlineStr"/>
+      <c r="J334" s="2" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
@@ -13350,6 +13773,7 @@
         </is>
       </c>
       <c r="I335" s="2" t="inlineStr"/>
+      <c r="J335" s="2" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
@@ -13389,6 +13813,7 @@
         </is>
       </c>
       <c r="I336" s="2" t="inlineStr"/>
+      <c r="J336" s="2" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
@@ -13432,6 +13857,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J337" s="2" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
@@ -13471,6 +13897,7 @@
         </is>
       </c>
       <c r="I338" s="2" t="inlineStr"/>
+      <c r="J338" s="2" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
@@ -13510,6 +13937,7 @@
         </is>
       </c>
       <c r="I339" s="2" t="inlineStr"/>
+      <c r="J339" s="2" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
@@ -13549,6 +13977,7 @@
         </is>
       </c>
       <c r="I340" s="2" t="inlineStr"/>
+      <c r="J340" s="2" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
@@ -13588,6 +14017,7 @@
         </is>
       </c>
       <c r="I341" s="2" t="inlineStr"/>
+      <c r="J341" s="2" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
@@ -13631,6 +14061,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J342" s="2" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
@@ -13670,6 +14101,11 @@
         </is>
       </c>
       <c r="I343" s="2" t="inlineStr"/>
+      <c r="J343" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
@@ -13705,6 +14141,7 @@
         </is>
       </c>
       <c r="I344" s="2" t="inlineStr"/>
+      <c r="J344" s="2" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
@@ -13740,6 +14177,7 @@
         </is>
       </c>
       <c r="I345" s="2" t="inlineStr"/>
+      <c r="J345" s="2" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
@@ -13779,6 +14217,7 @@
           <t>yes 2026-07-29 (read in full)</t>
         </is>
       </c>
+      <c r="J346" s="2" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
@@ -13814,6 +14253,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J347" s="2" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
@@ -13853,6 +14293,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J348" s="2" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
@@ -13896,6 +14337,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J349" s="2" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
@@ -13939,6 +14381,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J350" s="2" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
@@ -13978,6 +14421,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J351" s="2" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
@@ -14021,6 +14465,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J352" s="2" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
@@ -14064,6 +14509,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J353" s="2" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
@@ -14103,6 +14549,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J354" s="2" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
@@ -14146,6 +14593,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J355" s="2" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
@@ -14189,6 +14637,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J356" s="2" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
@@ -14232,6 +14681,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J357" s="2" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
@@ -14271,6 +14721,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J358" s="2" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
@@ -14310,6 +14761,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J359" s="2" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
@@ -14349,6 +14801,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J360" s="2" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
@@ -14392,6 +14845,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J361" s="2" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
@@ -14431,6 +14885,7 @@
         </is>
       </c>
       <c r="I362" s="2" t="inlineStr"/>
+      <c r="J362" s="2" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
@@ -14474,6 +14929,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J363" s="2" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
@@ -14513,6 +14969,7 @@
         </is>
       </c>
       <c r="I364" s="2" t="inlineStr"/>
+      <c r="J364" s="2" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
@@ -14552,6 +15009,7 @@
         </is>
       </c>
       <c r="I365" s="2" t="inlineStr"/>
+      <c r="J365" s="2" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
@@ -14591,6 +15049,7 @@
         </is>
       </c>
       <c r="I366" s="2" t="inlineStr"/>
+      <c r="J366" s="2" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
@@ -14630,6 +15089,7 @@
         </is>
       </c>
       <c r="I367" s="2" t="inlineStr"/>
+      <c r="J367" s="2" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
@@ -14673,6 +15133,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J368" s="2" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
@@ -14716,6 +15177,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J369" s="2" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
@@ -14759,6 +15221,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J370" s="2" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
@@ -14798,6 +15261,7 @@
         </is>
       </c>
       <c r="I371" s="2" t="inlineStr"/>
+      <c r="J371" s="2" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" s="2" t="inlineStr">
@@ -14837,6 +15301,7 @@
         </is>
       </c>
       <c r="I372" s="2" t="inlineStr"/>
+      <c r="J372" s="2" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
@@ -14876,6 +15341,7 @@
         </is>
       </c>
       <c r="I373" s="2" t="inlineStr"/>
+      <c r="J373" s="2" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
@@ -14915,6 +15381,7 @@
         </is>
       </c>
       <c r="I374" s="2" t="inlineStr"/>
+      <c r="J374" s="2" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
@@ -14954,6 +15421,7 @@
         </is>
       </c>
       <c r="I375" s="2" t="inlineStr"/>
+      <c r="J375" s="2" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
@@ -14993,6 +15461,7 @@
         </is>
       </c>
       <c r="I376" s="2" t="inlineStr"/>
+      <c r="J376" s="2" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
@@ -15032,6 +15501,7 @@
         </is>
       </c>
       <c r="I377" s="2" t="inlineStr"/>
+      <c r="J377" s="2" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
@@ -15067,6 +15537,7 @@
         </is>
       </c>
       <c r="I378" s="2" t="inlineStr"/>
+      <c r="J378" s="2" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
@@ -15102,6 +15573,7 @@
         </is>
       </c>
       <c r="I379" s="2" t="inlineStr"/>
+      <c r="J379" s="2" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
@@ -15137,6 +15609,7 @@
         </is>
       </c>
       <c r="I380" s="2" t="inlineStr"/>
+      <c r="J380" s="2" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
@@ -15172,6 +15645,7 @@
         </is>
       </c>
       <c r="I381" s="2" t="inlineStr"/>
+      <c r="J381" s="2" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
@@ -15207,6 +15681,11 @@
         </is>
       </c>
       <c r="I382" s="2" t="inlineStr"/>
+      <c r="J382" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="inlineStr">
@@ -15242,6 +15721,11 @@
         </is>
       </c>
       <c r="I383" s="2" t="inlineStr"/>
+      <c r="J383" s="2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">
@@ -15277,6 +15761,7 @@
         </is>
       </c>
       <c r="I384" s="2" t="inlineStr"/>
+      <c r="J384" s="2" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
@@ -15312,6 +15797,7 @@
         </is>
       </c>
       <c r="I385" s="2" t="inlineStr"/>
+      <c r="J385" s="2" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
@@ -15351,6 +15837,7 @@
         </is>
       </c>
       <c r="I386" s="2" t="inlineStr"/>
+      <c r="J386" s="2" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
@@ -15390,6 +15877,7 @@
         </is>
       </c>
       <c r="I387" s="2" t="inlineStr"/>
+      <c r="J387" s="2" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" s="2" t="inlineStr">
@@ -15425,6 +15913,7 @@
         </is>
       </c>
       <c r="I388" s="2" t="inlineStr"/>
+      <c r="J388" s="2" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" s="2" t="inlineStr">
@@ -15464,6 +15953,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J389" s="2" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
@@ -15499,6 +15989,7 @@
         </is>
       </c>
       <c r="I390" s="2" t="inlineStr"/>
+      <c r="J390" s="2" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" s="2" t="inlineStr">
@@ -15538,6 +16029,7 @@
           <t>yes 2026-07-29</t>
         </is>
       </c>
+      <c r="J391" s="2" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" s="2" t="inlineStr">
@@ -15573,6 +16065,7 @@
         </is>
       </c>
       <c r="I392" s="2" t="inlineStr"/>
+      <c r="J392" s="2" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" s="2" t="inlineStr">
@@ -15608,6 +16101,7 @@
         </is>
       </c>
       <c r="I393" s="2" t="inlineStr"/>
+      <c r="J393" s="2" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" s="2" t="inlineStr">
@@ -15643,6 +16137,7 @@
         </is>
       </c>
       <c r="I394" s="2" t="inlineStr"/>
+      <c r="J394" s="2" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">
@@ -15678,6 +16173,7 @@
         </is>
       </c>
       <c r="I395" s="2" t="inlineStr"/>
+      <c r="J395" s="2" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" s="2" t="inlineStr">
@@ -15713,6 +16209,7 @@
         </is>
       </c>
       <c r="I396" s="2" t="inlineStr"/>
+      <c r="J396" s="2" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
@@ -15748,6 +16245,7 @@
         </is>
       </c>
       <c r="I397" s="2" t="inlineStr"/>
+      <c r="J397" s="2" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
@@ -15783,6 +16281,7 @@
         </is>
       </c>
       <c r="I398" s="2" t="inlineStr"/>
+      <c r="J398" s="2" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" s="2" t="inlineStr">
@@ -15818,6 +16317,7 @@
         </is>
       </c>
       <c r="I399" s="2" t="inlineStr"/>
+      <c r="J399" s="2" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
@@ -15853,6 +16353,7 @@
         </is>
       </c>
       <c r="I400" s="2" t="inlineStr"/>
+      <c r="J400" s="2" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
@@ -15888,6 +16389,7 @@
         </is>
       </c>
       <c r="I401" s="2" t="inlineStr"/>
+      <c r="J401" s="2" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
@@ -15923,9 +16425,10 @@
         </is>
       </c>
       <c r="I402" s="2" t="inlineStr"/>
+      <c r="J402" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I402"/>
+  <autoFilter ref="A1:J402"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16563,14 +17066,12 @@
           <t>— Live paper-specific postulates</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>~15</t>
-        </is>
+      <c r="B11" s="6" t="n">
+        <v>15</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>of 24 Postulated rows: −6 Foundations meta-rows (about the axiom system), −3 discharged/definitional (P14→QuadraticStrain, P-GW-Saddle=naming, P-NonAbelian-Analogy→MS-II). The only per-domain knobs; some still shared (V5).</t>
+          <t>of 24 Postulated rows (see the 'Postulate' flag column on the Claims sheet): 15 live, 2 discharged (P14→QuadraticStrain, P-NonAbelian-Analogy→MS-II §2), 1 definitional-only (P-GW-Saddle, naming), 6 Foundations meta-rows. The live ones are the only per-domain knobs; some still shared (V5).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master: sharpen a0(z) prediction falsifier with the cH(z)-vs-c2sqrt(Lambda) discriminator (reverse-pass find; high-z RAR mildly favors ED's rising-with-z relation)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ED_TieredClaims_Master.xlsx
+++ b/ED_TieredClaims_Master.xlsx
@@ -1593,7 +1593,7 @@
       </c>
       <c r="E2" s="40" t="inlineStr">
         <is>
-          <t>departs from cH(z)/2pi. Only 031 §8.8 is data-confronted: MUSE-DARK III (A&amp;A 2026) ~30sigma evolution, ~8% local, edge of H(z); alpha=1 the decisive open number. Do NOT over-bank (direction won, exact rate tense)</t>
+          <t>departs from cH(z)/2pi. Only 031 §8.8 is data-confronted: MUSE-DARK III (A&amp;A 2026) ~30sigma evolution, ~8% local, edge of H(z); alpha=1 the decisive open number. Do NOT over-bank (direction won, exact rate tense) || DISCRIMINATOR (2026-08-02): a0=cH(z) [ED, RISES with z] vs a0=c2*sqrt(Lambda) [CONSTANT] coincide today but diverge with z; a0 following the sqrt(Lambda)-constant form rather than cH(z) refutes the ED relation. Recent high-z RAR literature (arXiv 2405.01841, 2504.20857) shows a MILD PREFERENCE for a0 rising with z -&gt; favors ED's cH(z) over the Lambda-tied form.</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="E46" s="41" t="inlineStr">
         <is>
-          <t>F3: MOND scale shown CONSTANT with z refutes it. First data (MUSE-DARK III, A&amp;A 2026) instead EXCLUDE constant a0 at ~30sigma (evolution confirmed); a robustly-confirmed rate incompatible with ~H(z) refutes the EXACT bet (data run faster), not the evolution</t>
+          <t>F3: MOND scale shown CONSTANT with z refutes it. First data (MUSE-DARK III, A&amp;A 2026) instead EXCLUDE constant a0 at ~30sigma (evolution confirmed); a robustly-confirmed rate incompatible with ~H(z) refutes the EXACT bet (data run faster), not the evolution || DISCRIMINATOR (2026-08-02): a0=cH(z) [ED, RISES with z] vs a0=c2*sqrt(Lambda) [CONSTANT] coincide today but diverge with z; a0 following the sqrt(Lambda)-constant form rather than cH(z) refutes the ED relation. Recent high-z RAR literature (arXiv 2405.01841, 2504.20857) shows a MILD PREFERENCE for a0 rising with z -&gt; favors ED's cH(z) over the Lambda-tied form.</t>
         </is>
       </c>
       <c r="F46" s="41" t="inlineStr">
@@ -13591,7 +13591,7 @@
       </c>
       <c r="E288" s="41" t="inlineStr">
         <is>
-          <t>departs from cH(z)/2pi. Only 031 §8.8 is data-confronted: MUSE-DARK III (A&amp;A 2026) ~30sigma evolution, ~8% local, edge of H(z); alpha=1 the decisive open number. Do NOT over-bank (direction won, exact rate tense)</t>
+          <t>departs from cH(z)/2pi. Only 031 §8.8 is data-confronted: MUSE-DARK III (A&amp;A 2026) ~30sigma evolution, ~8% local, edge of H(z); alpha=1 the decisive open number. Do NOT over-bank (direction won, exact rate tense) || DISCRIMINATOR (2026-08-02): a0=cH(z) [ED, RISES with z] vs a0=c2*sqrt(Lambda) [CONSTANT] coincide today but diverge with z; a0 following the sqrt(Lambda)-constant form rather than cH(z) refutes the ED relation. Recent high-z RAR literature (arXiv 2405.01841, 2504.20857) shows a MILD PREFERENCE for a0 rising with z -&gt; favors ED's cH(z) over the Lambda-tied form.</t>
         </is>
       </c>
       <c r="F288" s="41" t="n"/>

</xml_diff>